<commit_message>
feat: add Power BI dashboard layer with KPI-aligned DAX measures
</commit_message>
<xml_diff>
--- a/data/gold/data_catalog.xlsx
+++ b/data/gold/data_catalog.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jadul\desktop_data_engineering\Banking_Risk_Operations_Dashboard\data\gold\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4481FD55-0F44-42AD-8BA3-6F5AADF84867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9E6C5FA-E19C-41AC-8BBD-C52DFF094933}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="kpi_catalog" sheetId="1" r:id="rId1"/>
-    <sheet name="metric_definition" sheetId="2" r:id="rId2"/>
-    <sheet name="business_glossary" sheetId="3" r:id="rId3"/>
-    <sheet name="semantic_layer" sheetId="4" r:id="rId4"/>
+    <sheet name="dashboard_plan" sheetId="5" r:id="rId1"/>
+    <sheet name="kpi_catalog" sheetId="1" r:id="rId2"/>
+    <sheet name="metric_definition" sheetId="2" r:id="rId3"/>
+    <sheet name="business_glossary" sheetId="3" r:id="rId4"/>
+    <sheet name="semantic_layer" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="148">
   <si>
     <t>kpi_id</t>
   </si>
@@ -613,6 +614,93 @@
   </si>
   <si>
     <t>fact_transaction</t>
+  </si>
+  <si>
+    <t>dashboard_page</t>
+  </si>
+  <si>
+    <t>audience</t>
+  </si>
+  <si>
+    <t>business_questions</t>
+  </si>
+  <si>
+    <t>primary_kpis</t>
+  </si>
+  <si>
+    <t>analysis_dimensions</t>
+  </si>
+  <si>
+    <t>source_data</t>
+  </si>
+  <si>
+    <t>Executive Overview</t>
+  </si>
+  <si>
+    <t>Executives, Risk Teams</t>
+  </si>
+  <si>
+    <t>What is the overall fraud situation and financial exposure?</t>
+  </si>
+  <si>
+    <t>Total Transactions, Fraudulent Transactions, Fraud Rate, Fraud Exposure Amount, Fraud Exposure Rate</t>
+  </si>
+  <si>
+    <t>dim_time, dim_transaction_type</t>
+  </si>
+  <si>
+    <t>Fraud Operations Monitoring</t>
+  </si>
+  <si>
+    <t>Operations Managers, Fraud Investigators, Analysts</t>
+  </si>
+  <si>
+    <t>When does fraud occur and how does activity change over time?</t>
+  </si>
+  <si>
+    <t>Fraudulent Transactions, Fraud Rate, Flagged Fraud Transactions</t>
+  </si>
+  <si>
+    <t>Risk Analysis</t>
+  </si>
+  <si>
+    <t>Risk Teams, Compliance Teams, Analysts</t>
+  </si>
+  <si>
+    <t>Which transaction types and patterns create the highest fraud exposure?</t>
+  </si>
+  <si>
+    <t>Fraud Exposure Amount, Fraud Exposure Rate, Average Fraud Amount</t>
+  </si>
+  <si>
+    <t>dim_transaction_type, amount_range</t>
+  </si>
+  <si>
+    <t>Data Quality Monitoring</t>
+  </si>
+  <si>
+    <t>Analysts, Operations/Data Teams</t>
+  </si>
+  <si>
+    <t>Can the current data supporting the dashboard be trusted?</t>
+  </si>
+  <si>
+    <t>dq rule status, failed checks, transaction history</t>
+  </si>
+  <si>
+    <t>check_type (completeness, validity), status (PASS, FAIL), run_timestamp</t>
+  </si>
+  <si>
+    <t>gold.xlsx</t>
+  </si>
+  <si>
+    <t>KPI Validation</t>
+  </si>
+  <si>
+    <t>Technical validation</t>
+  </si>
+  <si>
+    <t>All 8 KPIs</t>
   </si>
 </sst>
 </file>
@@ -649,7 +737,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -657,11 +745,122 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -669,14 +868,244 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="32">
+  <dxfs count="55">
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -695,27 +1124,22 @@
         <scheme val="minor"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -734,15 +1158,90 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -762,15 +1261,71 @@
         <scheme val="minor"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -788,22 +1343,121 @@
         <name val="Arial Unicode MS"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -823,15 +1477,89 @@
         <scheme val="minor"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -849,19 +1577,116 @@
         <name val="Arial Unicode MS"/>
         <scheme val="none"/>
       </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -881,6 +1706,213 @@
         <scheme val="minor"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -896,60 +1928,70 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{9DA2BD9D-4B7B-43B9-AD7D-F34927F74A40}" name="Table2" displayName="Table2" ref="A1:G9" totalsRowShown="0" headerRowDxfId="31" dataDxfId="30">
-  <autoFilter ref="A1:G9" xr:uid="{9DA2BD9D-4B7B-43B9-AD7D-F34927F74A40}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{1473AFE9-A0BA-406B-B001-FAF37F7FBFD8}" name="kpi_id" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{2DF7C00F-E328-4948-B31E-CD5DE66A4571}" name="kpi_name" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{3F0B5F99-63C0-470B-B52A-3FE4F7D2A450}" name="business_definition" dataDxfId="27"/>
-    <tableColumn id="5" xr3:uid="{E3B765F5-2F42-4B68-AFD0-8E3E2D678B02}" name="source_columns" dataDxfId="26"/>
-    <tableColumn id="6" xr3:uid="{0554EBB9-B560-49F8-9693-0E827A825867}" name="aggregation" dataDxfId="25"/>
-    <tableColumn id="10" xr3:uid="{D233E88C-1D17-4C21-AB11-B823D00294F4}" name="stakeholders" dataDxfId="24"/>
-    <tableColumn id="11" xr3:uid="{BCDB67CF-A37D-4442-8D6B-BD76EFF2C412}" name="priority" dataDxfId="23"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{A4381767-F437-46DD-A3C4-18D4A7545610}" name="Table5" displayName="Table5" ref="A1:F6" totalsRowShown="0" headerRowDxfId="54" dataDxfId="52" headerRowBorderDxfId="53" tableBorderDxfId="51" totalsRowBorderDxfId="50">
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{53086735-911F-4828-8CE9-4742A234A47F}" name="dashboard_page" dataDxfId="49"/>
+    <tableColumn id="2" xr3:uid="{9068B6FD-7D1D-4169-A8BB-A5307C0B2559}" name="audience" dataDxfId="48"/>
+    <tableColumn id="3" xr3:uid="{9ECEF6A0-1CD7-44C3-89A0-700AC20EEBB1}" name="business_questions" dataDxfId="47"/>
+    <tableColumn id="4" xr3:uid="{0D73E923-4AC6-4B98-A8D5-812574D4EDF8}" name="primary_kpis" dataDxfId="46"/>
+    <tableColumn id="7" xr3:uid="{09D8C069-D1A9-4590-9C4E-331F4D007997}" name="analysis_dimensions" dataDxfId="45"/>
+    <tableColumn id="6" xr3:uid="{70109058-31EF-414A-B5D7-3E1B61A5FE42}" name="source_data" dataDxfId="44"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{FFF5F5B9-FEB0-42BB-B8B4-171D35A454F7}" name="Table3" displayName="Table3" ref="A1:H9" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
-  <autoFilter ref="A1:H9" xr:uid="{FFF5F5B9-FEB0-42BB-B8B4-171D35A454F7}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{24714AFA-E80A-490E-B5B9-E03F38F6562E}" name="kpi_id" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{C0DC9EDC-BD9B-4D0F-A0FC-8BAD4B0FA86A}" name="kpi_name" dataDxfId="19"/>
-    <tableColumn id="4" xr3:uid="{F172DAF9-9238-421E-925D-6725101559CE}" name="numerator" dataDxfId="18"/>
-    <tableColumn id="5" xr3:uid="{F39C91BE-3B7E-459B-92F8-884B4DF7DAE4}" name="denominator" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{33ECD701-E58F-4FCF-89A9-214031CCA9E5}" name="filter_condition" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{AA57093E-370E-4495-ABDF-D7D67A84AF0D}" name="calculation_logic" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{B81970FB-8D8C-4696-8039-3F30637506D1}" name="zero_denominator_handling" dataDxfId="14"/>
-    <tableColumn id="9" xr3:uid="{57798366-DEBF-4907-B427-35B1674EA69B}" name="format" dataDxfId="13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{9DA2BD9D-4B7B-43B9-AD7D-F34927F74A40}" name="Table2" displayName="Table2" ref="A1:G9" totalsRowShown="0" headerRowDxfId="43" dataDxfId="41" headerRowBorderDxfId="42" tableBorderDxfId="40" totalsRowBorderDxfId="39">
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{1473AFE9-A0BA-406B-B001-FAF37F7FBFD8}" name="kpi_id" dataDxfId="38"/>
+    <tableColumn id="2" xr3:uid="{2DF7C00F-E328-4948-B31E-CD5DE66A4571}" name="kpi_name" dataDxfId="37"/>
+    <tableColumn id="3" xr3:uid="{3F0B5F99-63C0-470B-B52A-3FE4F7D2A450}" name="business_definition" dataDxfId="36"/>
+    <tableColumn id="5" xr3:uid="{E3B765F5-2F42-4B68-AFD0-8E3E2D678B02}" name="source_columns" dataDxfId="35"/>
+    <tableColumn id="6" xr3:uid="{0554EBB9-B560-49F8-9693-0E827A825867}" name="aggregation" dataDxfId="34"/>
+    <tableColumn id="10" xr3:uid="{D233E88C-1D17-4C21-AB11-B823D00294F4}" name="stakeholders" dataDxfId="33"/>
+    <tableColumn id="11" xr3:uid="{BCDB67CF-A37D-4442-8D6B-BD76EFF2C412}" name="priority" dataDxfId="32"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F17627FD-4ABD-4A53-81D3-A851884E939A}" name="Table4" displayName="Table4" ref="A1:C11" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
-  <autoFilter ref="A1:C11" xr:uid="{F17627FD-4ABD-4A53-81D3-A851884E939A}"/>
-  <tableColumns count="3">
-    <tableColumn id="2" xr3:uid="{A7C01615-2FA4-4FDA-8F1C-1542FBA6092E}" name="term" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{B3BF12D5-A599-4218-8A7C-22C9615F8E77}" name="definition" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{057D2D3D-F8C5-4B47-9B4C-41A7D2474A75}" name="related_columns" dataDxfId="8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{FFF5F5B9-FEB0-42BB-B8B4-171D35A454F7}" name="Table3" displayName="Table3" ref="A1:H9" totalsRowShown="0" headerRowDxfId="31" dataDxfId="29" headerRowBorderDxfId="30" tableBorderDxfId="28" totalsRowBorderDxfId="27">
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{24714AFA-E80A-490E-B5B9-E03F38F6562E}" name="kpi_id" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{C0DC9EDC-BD9B-4D0F-A0FC-8BAD4B0FA86A}" name="kpi_name" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{F172DAF9-9238-421E-925D-6725101559CE}" name="numerator" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{F39C91BE-3B7E-459B-92F8-884B4DF7DAE4}" name="denominator" dataDxfId="23"/>
+    <tableColumn id="6" xr3:uid="{33ECD701-E58F-4FCF-89A9-214031CCA9E5}" name="filter_condition" dataDxfId="22"/>
+    <tableColumn id="7" xr3:uid="{AA57093E-370E-4495-ABDF-D7D67A84AF0D}" name="calculation_logic" dataDxfId="21"/>
+    <tableColumn id="8" xr3:uid="{B81970FB-8D8C-4696-8039-3F30637506D1}" name="zero_denominator_handling" dataDxfId="20"/>
+    <tableColumn id="9" xr3:uid="{57798366-DEBF-4907-B427-35B1674EA69B}" name="format" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{65B7B6B4-00D1-47B3-A5AA-88A4E75C35C4}" name="Table1" displayName="Table1" ref="A1:F4" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
-  <autoFilter ref="A1:F4" xr:uid="{65B7B6B4-00D1-47B3-A5AA-88A4E75C35C4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{F17627FD-4ABD-4A53-81D3-A851884E939A}" name="Table4" displayName="Table4" ref="A1:C11" totalsRowShown="0" headerRowDxfId="18" dataDxfId="16" headerRowBorderDxfId="17" tableBorderDxfId="15" totalsRowBorderDxfId="14">
+  <tableColumns count="3">
+    <tableColumn id="2" xr3:uid="{A7C01615-2FA4-4FDA-8F1C-1542FBA6092E}" name="term" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{B3BF12D5-A599-4218-8A7C-22C9615F8E77}" name="definition" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{057D2D3D-F8C5-4B47-9B4C-41A7D2474A75}" name="related_columns" dataDxfId="11"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{65B7B6B4-00D1-47B3-A5AA-88A4E75C35C4}" name="Table1" displayName="Table1" ref="A1:F4" totalsRowShown="0" headerRowDxfId="10" dataDxfId="8" headerRowBorderDxfId="9" tableBorderDxfId="7" totalsRowBorderDxfId="6">
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{4354B1AF-CBBF-40DA-846F-5F02BB2EF54E}" name="entity" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{2799A860-02C1-4C17-A631-E9130F36AAB4}" name="entity_type" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{6BBE34C7-2507-43D8-98F1-6EB244E8E76C}" name="business_purpose" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{E6AD72CA-BD8A-46C0-8B8E-5B0C001151B5}" name="key" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{268BAFB9-1C30-42F2-9D8E-CDA311B8E768}" name="metrics_or_attributes" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{3771446C-3650-47E2-97F3-1F403BF532CF}" name="relationships" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{4354B1AF-CBBF-40DA-846F-5F02BB2EF54E}" name="entity" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{2799A860-02C1-4C17-A631-E9130F36AAB4}" name="entity_type" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{6BBE34C7-2507-43D8-98F1-6EB244E8E76C}" name="business_purpose" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{E6AD72CA-BD8A-46C0-8B8E-5B0C001151B5}" name="key" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{268BAFB9-1C30-42F2-9D8E-CDA311B8E768}" name="metrics_or_attributes" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{3771446C-3650-47E2-97F3-1F403BF532CF}" name="relationships" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1217,225 +2259,169 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D6CC770B-C139-4985-B40A-B22FC3DE0509}">
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="70.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="60.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.7109375" style="3" customWidth="1"/>
+    <col min="4" max="4" width="30.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.5703125" style="3" customWidth="1"/>
+    <col min="6" max="6" width="19.85546875" style="3" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15" customHeight="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="15" customHeight="1">
-      <c r="A2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="15" customHeight="1">
-      <c r="A3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="15" customHeight="1">
-      <c r="A4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="15" customHeight="1">
-      <c r="A5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="15" customHeight="1">
-      <c r="A6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="15" customHeight="1">
-      <c r="A7" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="15" customHeight="1">
-      <c r="A8" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="15" customHeight="1">
-      <c r="A9" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>24</v>
-      </c>
+    <row r="1" spans="1:6" ht="15">
+      <c r="A1" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="15">
+      <c r="A2" s="23" t="s">
+        <v>145</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="60">
+      <c r="A3" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="45">
+      <c r="A5" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="75">
+      <c r="A6" s="12" t="s">
+        <v>139</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="30" customHeight="1">
+      <c r="A8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="F8" s="1"/>
+    </row>
+    <row r="9" spans="1:6" ht="30" customHeight="1">
+      <c r="A9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="F9" s="2"/>
+    </row>
+    <row r="10" spans="1:6" ht="30" customHeight="1">
+      <c r="A10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2"/>
+      <c r="F10" s="2"/>
+    </row>
+    <row r="11" spans="1:6" ht="30" customHeight="1">
+      <c r="A11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="F11" s="2"/>
+    </row>
+    <row r="12" spans="1:6" ht="30" customHeight="1">
+      <c r="A12" s="2"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2"/>
+      <c r="F12" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1446,252 +2432,223 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A43D731-AB88-451D-83D1-4608580C9B59}">
-  <dimension ref="A1:H9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="37.7109375" customWidth="1"/>
-    <col min="6" max="6" width="51.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="38.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.140625" customWidth="1"/>
+    <col min="2" max="3" width="25.7109375" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15" customHeight="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="15" customHeight="1">
-      <c r="A2" s="2" t="s">
+      <c r="C1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="45">
+      <c r="A2" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="15" customHeight="1">
-      <c r="A3" s="2" t="s">
+      <c r="C2" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="45">
+      <c r="A3" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="15" customHeight="1">
-      <c r="A4" s="2" t="s">
+      <c r="C3" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="45">
+      <c r="A4" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="15" customHeight="1">
-      <c r="A5" s="2" t="s">
+      <c r="C4" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="45">
+      <c r="A5" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="15" customHeight="1">
-      <c r="A6" s="2" t="s">
+      <c r="C5" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="45">
+      <c r="A6" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="15" customHeight="1">
-      <c r="A7" s="2" t="s">
+      <c r="C6" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="60">
+      <c r="A7" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="15" customHeight="1">
-      <c r="A8" s="2" t="s">
+      <c r="C7" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="30">
+      <c r="A8" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="15" customHeight="1">
-      <c r="A9" s="2" t="s">
+      <c r="C8" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="45">
+      <c r="A9" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>12</v>
+      <c r="C9" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -1703,133 +2660,391 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A43D731-AB88-451D-83D1-4608580C9B59}">
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr defaultRowHeight="30" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.5703125" customWidth="1"/>
+    <col min="6" max="6" width="21.42578125" customWidth="1"/>
+    <col min="7" max="7" width="17.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="45">
+      <c r="A4" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="27.75">
+      <c r="A6" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="51">
+      <c r="A7" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="45">
+      <c r="A8" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="F8" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="42.75">
+      <c r="A9" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D624B80-9DC1-45BA-9301-0995A248DBF6}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="24.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="104.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="60.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15" customHeight="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="6" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15" customHeight="1">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:3">
+      <c r="A2" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="19" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15" customHeight="1">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:3" ht="30">
+      <c r="A3" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="19" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15" customHeight="1">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:3">
+      <c r="A4" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="19" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15" customHeight="1">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:3" ht="30">
+      <c r="A5" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="19" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15" customHeight="1">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:3" ht="30">
+      <c r="A6" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="19" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15" customHeight="1">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:3" ht="30">
+      <c r="A7" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="19" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15" customHeight="1">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:3">
+      <c r="A8" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="19" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15" customHeight="1">
-      <c r="A9" s="2" t="s">
+    <row r="9" spans="1:3">
+      <c r="A9" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="19" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15" customHeight="1">
-      <c r="A10" s="2" t="s">
+    <row r="10" spans="1:3" ht="30">
+      <c r="A10" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="19" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15" customHeight="1">
-      <c r="A11" s="2" t="s">
+    <row r="11" spans="1:3" ht="30">
+      <c r="A11" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="20" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1841,96 +3056,96 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6C87987-72C0-4295-BEED-353AA8D1FFBF}">
   <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="20.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="65.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="52" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" customWidth="1"/>
+    <col min="5" max="5" width="32.140625" customWidth="1"/>
     <col min="6" max="6" width="41.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" customHeight="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6">
+      <c r="A1" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="6" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15" customHeight="1">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:6" ht="30">
+      <c r="A2" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="15" t="s">
         <v>103</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="16" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15" customHeight="1">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:6" ht="30">
+      <c r="A3" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="16" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15" customHeight="1">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:6" ht="30">
+      <c r="A4" s="22" t="s">
         <v>114</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="17" t="s">
         <v>109</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="17" t="s">
         <v>115</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="17" t="s">
         <v>116</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="18" t="s">
         <v>113</v>
       </c>
     </row>

</xml_diff>